<commit_message>
updated files for travel
</commit_message>
<xml_diff>
--- a/updated_2025/data/imf_groupings.xlsx
+++ b/updated_2025/data/imf_groupings.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eclow\Documents\GitHub\cab-persistency\updated_2025\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4BD168B5-179F-4DBC-8D3C-5970C5155BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84038905-E43C-4E73-A913-A9B3D617CF05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-276" windowWidth="23256" windowHeight="12456" xr2:uid="{C53DD6F0-3390-4672-8BBE-72429E7B7539}"/>
+    <workbookView xWindow="-23148" yWindow="-2016" windowWidth="23256" windowHeight="12456" xr2:uid="{C53DD6F0-3390-4672-8BBE-72429E7B7539}"/>
   </bookViews>
   <sheets>
     <sheet name="imf_groupings" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">imf_groupings!$A$1:$U$200</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -2788,7 +2791,7 @@
         <v>0</v>
       </c>
       <c r="U19">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.3">
@@ -3112,6 +3115,9 @@
       <c r="T24">
         <v>0</v>
       </c>
+      <c r="U24">
+        <v>963</v>
+      </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
@@ -4589,6 +4595,9 @@
       <c r="T47">
         <v>0</v>
       </c>
+      <c r="U47">
+        <v>960</v>
+      </c>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
@@ -6598,6 +6607,9 @@
       <c r="T78">
         <v>0</v>
       </c>
+      <c r="U78">
+        <v>532</v>
+      </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
@@ -8344,6 +8356,9 @@
       <c r="T105">
         <v>0</v>
       </c>
+      <c r="U105">
+        <v>137</v>
+      </c>
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
@@ -8468,6 +8483,9 @@
       <c r="T107">
         <v>0</v>
       </c>
+      <c r="U107">
+        <v>962</v>
+      </c>
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
@@ -9369,6 +9387,9 @@
       <c r="T121">
         <v>0</v>
       </c>
+      <c r="U121">
+        <v>943</v>
+      </c>
     </row>
     <row r="122" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
@@ -9948,6 +9969,9 @@
       <c r="T130">
         <v>0</v>
       </c>
+      <c r="U130">
+        <v>138</v>
+      </c>
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
@@ -11174,9 +11198,6 @@
       <c r="T149">
         <v>0</v>
       </c>
-      <c r="U149">
-        <v>922</v>
-      </c>
     </row>
     <row r="150" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
@@ -11239,6 +11260,9 @@
       <c r="T150">
         <v>1</v>
       </c>
+      <c r="U150">
+        <v>922</v>
+      </c>
     </row>
     <row r="151" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
@@ -11883,6 +11907,9 @@
       <c r="T160">
         <v>0</v>
       </c>
+      <c r="U160">
+        <v>936</v>
+      </c>
     </row>
     <row r="161" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
@@ -11945,6 +11972,9 @@
       <c r="T161">
         <v>0</v>
       </c>
+      <c r="U161">
+        <v>961</v>
+      </c>
     </row>
     <row r="162" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
@@ -12840,6 +12870,9 @@
       <c r="T175">
         <v>0</v>
       </c>
+      <c r="U175">
+        <v>528</v>
+      </c>
     </row>
     <row r="176" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
@@ -13416,6 +13449,9 @@
       <c r="T184">
         <v>0</v>
       </c>
+      <c r="U184">
+        <v>186</v>
+      </c>
     </row>
     <row r="185" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
@@ -14193,6 +14229,9 @@
       <c r="T196">
         <v>0</v>
       </c>
+      <c r="U196">
+        <v>582</v>
+      </c>
     </row>
     <row r="197" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
@@ -14449,6 +14488,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:U200" xr:uid="{7AF9A065-4918-4B64-969D-4B00887BD2FD}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U200">
     <sortCondition ref="A91:A200"/>
   </sortState>

</xml_diff>